<commit_message>
added screenshots, hooks, POM ect
</commit_message>
<xml_diff>
--- a/Playwright_master.xlsx
+++ b/Playwright_master.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="CommonError&amp;sloution" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="154">
   <si>
     <t xml:space="preserve">Error </t>
   </si>
@@ -298,12 +298,368 @@
   <si>
     <t>pease check input formate matches with field formate</t>
   </si>
+  <si>
+    <t>Date()</t>
+  </si>
+  <si>
+    <t>used to get current date and time</t>
+  </si>
+  <si>
+    <t>.getDate()</t>
+  </si>
+  <si>
+    <t>to get current day</t>
+  </si>
+  <si>
+    <t>.getMonth()</t>
+  </si>
+  <si>
+    <t>get current month</t>
+  </si>
+  <si>
+    <t>.getFullYear()</t>
+  </si>
+  <si>
+    <t>get current year</t>
+  </si>
+  <si>
+    <t>padStart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">used to get validation of full lengh </t>
+  </si>
+  <si>
+    <r>
+      <t>month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF795E26"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>padStart</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF098658"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>'0'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>while(true)</t>
+  </si>
+  <si>
+    <t>runs continously until condition meets</t>
+  </si>
+  <si>
+    <t>to click on specific locator</t>
+  </si>
+  <si>
+    <t>locator.Click()</t>
+  </si>
+  <si>
+    <t>locator.Click({button:'right'})</t>
+  </si>
+  <si>
+    <t>to right click</t>
+  </si>
+  <si>
+    <t>page.click("locator",{button:'right'})</t>
+  </si>
+  <si>
+    <t>page.locator.dblclick();</t>
+  </si>
+  <si>
+    <t>to double click</t>
+  </si>
+  <si>
+    <t>locator.hover();</t>
+  </si>
+  <si>
+    <t>to mouse hover</t>
+  </si>
+  <si>
+    <t>page.dragAndDrop(source locator,target locator)</t>
+  </si>
+  <si>
+    <t>to drag and drop</t>
+  </si>
+  <si>
+    <t>page.locator().dragto()</t>
+  </si>
+  <si>
+    <t>page.mouse.wheel(pixel)</t>
+  </si>
+  <si>
+    <t>page.locator().focus()</t>
+  </si>
+  <si>
+    <t>to focus on element</t>
+  </si>
+  <si>
+    <t>page.keyboard</t>
+  </si>
+  <si>
+    <t>used to work with keyboard</t>
+  </si>
+  <si>
+    <t>page.keyboared.press("btn to click" )</t>
+  </si>
+  <si>
+    <t>press enter ofr shift</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Error: keyboard.press: Unknown key: "control"</t>
+  </si>
+  <si>
+    <t>playwright is case sensitive "Control" is correct</t>
+  </si>
+  <si>
+    <t>page.keyboard.down("Shift") /up</t>
+  </si>
+  <si>
+    <t>to hold down /up key</t>
+  </si>
+  <si>
+    <t>to upload file single/multiple --&gt; tag input attribute type =file</t>
+  </si>
+  <si>
+    <t>if mutiple attribute is there then only we can upload multiple file</t>
+  </si>
+  <si>
+    <t>path.join</t>
+  </si>
+  <si>
+    <t>make sure that path works correctly across diff os , no need to give / for path</t>
+  </si>
+  <si>
+    <t>page.setInputFiles("locator", filepath)</t>
+  </si>
+  <si>
+    <t>Error: ENOENT: no such file or directory, 
+stat 'C:\Users\admin\Desktop\Playwright_Study\tests\demo\data\uploads\one.txt'</t>
+  </si>
+  <si>
+    <t>while uploadig file by setInputFile if path incorrect then shows this error , please check file/folder path</t>
+  </si>
+  <si>
+    <r>
+      <t>path</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF795E26"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>join</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF001080"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>process</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF795E26"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>cwd</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>(),"data","uploads","one.txt"));</t>
+    </r>
+  </si>
+  <si>
+    <t>give file opth using , seperator</t>
+  </si>
+  <si>
+    <t>TimeoutError: page.setInputFiles: Timeout 10000ms exceeded.</t>
+  </si>
+  <si>
+    <t>if trying to handle correct locator inside frame without considering frame</t>
+  </si>
+  <si>
+    <t>Date.now()</t>
+  </si>
+  <si>
+    <t>used to identify screenshots uniquely without overwrite</t>
+  </si>
+  <si>
+    <t>PA</t>
+  </si>
+  <si>
+    <t>1st month cal</t>
+  </si>
+  <si>
+    <t>procng fee</t>
+  </si>
+  <si>
+    <t>igst</t>
+  </si>
+  <si>
+    <t>EMI</t>
+  </si>
+  <si>
+    <t>EMI INT</t>
+  </si>
+  <si>
+    <t>Interest(16%)</t>
+  </si>
+  <si>
+    <t>6 months cal</t>
+  </si>
+  <si>
+    <t>.describe</t>
+  </si>
+  <si>
+    <t>we can group or organize test cases</t>
+  </si>
+  <si>
+    <t>Expect "toBeVisible" with timeout 5000ms</t>
+  </si>
+  <si>
+    <t>element not loaded I 5 sec  , increase expect timeout / check locator is correct</t>
+  </si>
+  <si>
+    <t>.toHaveText()</t>
+  </si>
+  <si>
+    <t>complete match</t>
+  </si>
+  <si>
+    <t>toContainText()</t>
+  </si>
+  <si>
+    <t>partial match</t>
+  </si>
+  <si>
+    <t>Error: locator.click: Unexpected token "&amp;" while parsing css selector "Alerts, Frame &amp; Windows". Did you mean to CSS.escape it?</t>
+  </si>
+  <si>
+    <t>please check for correct locator</t>
+  </si>
+  <si>
+    <t>protected Page : page</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> this class is use this page object and classes inherite use this</t>
+  </si>
+  <si>
+    <t>it is the special function which runs automatically when you create object of class</t>
+  </si>
+  <si>
+    <t>constructor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">extends </t>
+  </si>
+  <si>
+    <t>use property and methods of specific class</t>
+  </si>
+  <si>
+    <t>If child class has constructor it should pass perent class constructor</t>
+  </si>
+  <si>
+    <t>validation only is in test case</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -341,16 +697,54 @@
       <name val="Courier New"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0070C1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF098658"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF001080"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -358,11 +752,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -370,13 +779,34 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -678,7 +1108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="41.28515625" customWidth="1"/>
@@ -713,7 +1143,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>63</v>
       </c>
       <c r="C4" t="s">
@@ -734,6 +1164,46 @@
       </c>
       <c r="C6" t="s">
         <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>124</v>
+      </c>
+      <c r="C9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C10" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -784,14 +1254,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.140625" customWidth="1"/>
-    <col min="5" max="5" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -920,7 +1391,7 @@
       <c r="B8" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -931,7 +1402,7 @@
       <c r="B9" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="3"/>
+      <c r="C9" s="7"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
@@ -989,7 +1460,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>56</v>
       </c>
@@ -997,7 +1468,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>55</v>
       </c>
@@ -1005,7 +1476,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" ht="60" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>59</v>
       </c>
@@ -1013,15 +1484,15 @@
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>65</v>
       </c>
@@ -1029,7 +1500,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>67</v>
       </c>
@@ -1037,7 +1508,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>69</v>
       </c>
@@ -1045,7 +1516,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>70</v>
       </c>
@@ -1053,7 +1524,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>73</v>
       </c>
@@ -1061,9 +1532,391 @@
         <v>74</v>
       </c>
     </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>81</v>
+      </c>
+      <c r="C27" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B30" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" t="s">
+        <v>88</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>90</v>
+      </c>
+      <c r="C31" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>93</v>
+      </c>
+      <c r="C32" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>94</v>
+      </c>
+      <c r="C33" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>99</v>
+      </c>
+      <c r="C36" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
+        <v>101</v>
+      </c>
+      <c r="C37" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>103</v>
+      </c>
+      <c r="C38" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>107</v>
+      </c>
+      <c r="C41" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B42" t="s">
+        <v>109</v>
+      </c>
+      <c r="C42" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
+        <v>113</v>
+      </c>
+      <c r="C43" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>119</v>
+      </c>
+      <c r="C44" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C45" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>117</v>
+      </c>
+      <c r="C46" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B47" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C47" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>126</v>
+      </c>
+      <c r="C48" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>136</v>
+      </c>
+      <c r="C49" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>140</v>
+      </c>
+      <c r="C50" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>142</v>
+      </c>
+      <c r="C51" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>146</v>
+      </c>
+      <c r="C52" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>149</v>
+      </c>
+      <c r="C53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>150</v>
+      </c>
+      <c r="C54" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C55" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C56" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C57" s="6"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="6"/>
+      <c r="F57" s="6"/>
+      <c r="G57" s="6"/>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C59" s="6"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="F59" s="12"/>
+      <c r="G59" s="6"/>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="F60" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="G60" s="6"/>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C61" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="D61" s="12"/>
+      <c r="E61" s="10">
+        <v>7253</v>
+      </c>
+      <c r="F61" s="10">
+        <v>980</v>
+      </c>
+      <c r="G61" s="6"/>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C62" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D62" s="10">
+        <v>299</v>
+      </c>
+      <c r="E62" s="10">
+        <v>7350</v>
+      </c>
+      <c r="F62" s="10">
+        <v>503</v>
+      </c>
+      <c r="G62" s="6"/>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C63" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="D63" s="10">
+        <v>53.82</v>
+      </c>
+      <c r="E63" s="10">
+        <v>7448</v>
+      </c>
+      <c r="F63" s="10">
+        <v>405</v>
+      </c>
+      <c r="G63" s="6"/>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C64" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D64" s="10">
+        <v>7253</v>
+      </c>
+      <c r="E64" s="10">
+        <v>7547</v>
+      </c>
+      <c r="F64" s="10">
+        <v>306</v>
+      </c>
+      <c r="G64" s="6"/>
+    </row>
+    <row r="65" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C65" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D65" s="10">
+        <v>980</v>
+      </c>
+      <c r="E65" s="10">
+        <v>7648</v>
+      </c>
+      <c r="F65" s="10">
+        <v>205</v>
+      </c>
+      <c r="G65" s="6"/>
+    </row>
+    <row r="66" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C66" s="6"/>
+      <c r="D66" s="9">
+        <f>SUM(D62:D65)</f>
+        <v>8585.82</v>
+      </c>
+      <c r="E66" s="10">
+        <v>7750</v>
+      </c>
+      <c r="F66" s="10">
+        <v>103</v>
+      </c>
+      <c r="G66" s="6"/>
+    </row>
+    <row r="67" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C67" s="6"/>
+      <c r="D67" s="6"/>
+      <c r="E67" s="11">
+        <f>SUM(E61:E66)</f>
+        <v>44996</v>
+      </c>
+      <c r="F67" s="11">
+        <f>SUM(F61:F66)</f>
+        <v>2502</v>
+      </c>
+      <c r="G67" s="8">
+        <f>E67+F67</f>
+        <v>47498</v>
+      </c>
+    </row>
+    <row r="68" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C68" s="6"/>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6"/>
+      <c r="F68" s="6"/>
+      <c r="G68" s="6"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="E59:F59"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add new test cases and helper functions for Playwright automation
- Created multiple test files for various functionalities including date picker, dropdowns, checkboxes, and assertions.
- Implemented helper functions for taking screenshots during tests.
- Added hooks for attaching screenshots on test failures.
- Included logical programs for palindrome checking.
- practice of palywrite concepts
</commit_message>
<xml_diff>
--- a/Playwright_master.xlsx
+++ b/Playwright_master.xlsx
@@ -10,13 +10,14 @@
     <sheet name="CommonError&amp;sloution" sheetId="1" r:id="rId1"/>
     <sheet name="Installed&amp;use" sheetId="2" r:id="rId2"/>
     <sheet name="Concepts&amp;Use" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="184">
   <si>
     <t xml:space="preserve">Error </t>
   </si>
@@ -653,6 +654,103 @@
   </si>
   <si>
     <t>validation only is in test case</t>
+  </si>
+  <si>
+    <t>npm install @faker-js/faker</t>
+  </si>
+  <si>
+    <t>used to generate random dynamic data</t>
+  </si>
+  <si>
+    <t>npm install openai dotenv</t>
+  </si>
+  <si>
+    <t>install open ai library to communicate ai model</t>
+  </si>
+  <si>
+    <t>^ - not \d - digit /g globally</t>
+  </si>
+  <si>
+    <t>regular expression "[^\d]/g"</t>
+  </si>
+  <si>
+    <t>.innerText()</t>
+  </si>
+  <si>
+    <t>get visible text</t>
+  </si>
+  <si>
+    <t>Idempotent requests -Put,Patch, Delete</t>
+  </si>
+  <si>
+    <t>server not changes as request is more than one</t>
+  </si>
+  <si>
+    <t>Api</t>
+  </si>
+  <si>
+    <t>fakeapi.com</t>
+  </si>
+  <si>
+    <t>dummyjson.com</t>
+  </si>
+  <si>
+    <t>page.locator().inputValue();</t>
+  </si>
+  <si>
+    <t>store it in variable to find text box deaault vale</t>
+  </si>
+  <si>
+    <t>Promise {
+  &lt;pending&gt;,
+  [Symbol(async_id_symbol)]: 34343,
+  [Symbol(trigger_async_id_symbol)]: 16314,
+  [Symbol(kResourceStore)]: undefined
+}</t>
+  </si>
+  <si>
+    <t>Print async playwright operation without await</t>
+  </si>
+  <si>
+    <t>Nullish Coalescing Operator (??)</t>
+  </si>
+  <si>
+    <t>0 is valid,
+empty string is valid,
+false is valid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">logical </t>
+  </si>
+  <si>
+    <t>UI dev Guide</t>
+  </si>
+  <si>
+    <t>Playwright</t>
+  </si>
+  <si>
+    <t>script and execute</t>
+  </si>
+  <si>
+    <t>step by step automation</t>
+  </si>
+  <si>
+    <t>How to use programming inautomation</t>
+  </si>
+  <si>
+    <t>npm install -g newman</t>
+  </si>
+  <si>
+    <t>used to execute postman using cli or cicd</t>
+  </si>
+  <si>
+    <t>webTechTalk</t>
+  </si>
+  <si>
+    <t>find all matching elements with this locator</t>
+  </si>
+  <si>
+    <t>page.$$</t>
   </si>
 </sst>
 </file>
@@ -789,9 +887,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -802,6 +897,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1108,7 +1206,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="41.28515625" customWidth="1"/>
@@ -1206,6 +1304,14 @@
         <v>145</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C12" t="s">
+        <v>170</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1213,7 +1319,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
@@ -1245,6 +1351,39 @@
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C4" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C6" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -1391,7 +1530,7 @@
       <c r="B8" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="11" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1402,7 +1541,7 @@
       <c r="B9" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="7"/>
+      <c r="C9" s="11"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
@@ -1476,7 +1615,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" ht="210" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>59</v>
       </c>
@@ -1769,140 +1908,59 @@
       </c>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="6"/>
+      <c r="B57" t="s">
+        <v>159</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>158</v>
+      </c>
       <c r="D57" s="6"/>
       <c r="E57" s="6"/>
       <c r="F57" s="6"/>
       <c r="G57" s="6"/>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C58" s="6"/>
+      <c r="B58" t="s">
+        <v>160</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>161</v>
+      </c>
       <c r="D58" s="6"/>
       <c r="E58" s="6"/>
       <c r="F58" s="6"/>
       <c r="G58" s="6"/>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C59" s="6"/>
-      <c r="D59" s="6"/>
-      <c r="E59" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="F59" s="12"/>
-      <c r="G59" s="6"/>
+      <c r="B59" t="s">
+        <v>162</v>
+      </c>
+      <c r="C59" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C60" s="6"/>
-      <c r="D60" s="6"/>
-      <c r="E60" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="F60" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="G60" s="6"/>
-    </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C61" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="D61" s="12"/>
-      <c r="E61" s="10">
-        <v>7253</v>
-      </c>
-      <c r="F61" s="10">
-        <v>980</v>
-      </c>
-      <c r="G61" s="6"/>
+      <c r="B60" t="s">
+        <v>167</v>
+      </c>
+      <c r="C60" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>171</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C62" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="D62" s="10">
-        <v>299</v>
-      </c>
-      <c r="E62" s="10">
-        <v>7350</v>
-      </c>
-      <c r="F62" s="10">
-        <v>503</v>
-      </c>
-      <c r="G62" s="6"/>
-    </row>
-    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C63" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="D63" s="10">
-        <v>53.82</v>
-      </c>
-      <c r="E63" s="10">
-        <v>7448</v>
-      </c>
-      <c r="F63" s="10">
-        <v>405</v>
-      </c>
-      <c r="G63" s="6"/>
-    </row>
-    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C64" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D64" s="10">
-        <v>7253</v>
-      </c>
-      <c r="E64" s="10">
-        <v>7547</v>
-      </c>
-      <c r="F64" s="10">
-        <v>306</v>
-      </c>
-      <c r="G64" s="6"/>
-    </row>
-    <row r="65" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C65" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="D65" s="10">
-        <v>980</v>
-      </c>
-      <c r="E65" s="10">
-        <v>7648</v>
-      </c>
-      <c r="F65" s="10">
-        <v>205</v>
-      </c>
-      <c r="G65" s="6"/>
-    </row>
-    <row r="66" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C66" s="6"/>
-      <c r="D66" s="9">
-        <f>SUM(D62:D65)</f>
-        <v>8585.82</v>
-      </c>
-      <c r="E66" s="10">
-        <v>7750</v>
-      </c>
-      <c r="F66" s="10">
-        <v>103</v>
-      </c>
-      <c r="G66" s="6"/>
-    </row>
-    <row r="67" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C67" s="6"/>
-      <c r="D67" s="6"/>
-      <c r="E67" s="11">
-        <f>SUM(E61:E66)</f>
-        <v>44996</v>
-      </c>
-      <c r="F67" s="11">
-        <f>SUM(F61:F66)</f>
-        <v>2502</v>
-      </c>
-      <c r="G67" s="8">
-        <f>E67+F67</f>
-        <v>47498</v>
+      <c r="B62" t="s">
+        <v>183</v>
+      </c>
+      <c r="C62" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="68" spans="3:7" x14ac:dyDescent="0.25">
@@ -1913,12 +1971,188 @@
       <c r="G68" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="1">
     <mergeCell ref="C8:C9"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="E59:F59"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="12"/>
+      <c r="E1" s="6"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E2" s="6"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="12"/>
+      <c r="C3" s="9">
+        <v>7253</v>
+      </c>
+      <c r="D3" s="9">
+        <v>980</v>
+      </c>
+      <c r="E3" s="6"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="9">
+        <v>299</v>
+      </c>
+      <c r="C4" s="9">
+        <v>7350</v>
+      </c>
+      <c r="D4" s="9">
+        <v>503</v>
+      </c>
+      <c r="E4" s="6"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" s="9">
+        <v>53.82</v>
+      </c>
+      <c r="C5" s="9">
+        <v>7448</v>
+      </c>
+      <c r="D5" s="9">
+        <v>405</v>
+      </c>
+      <c r="E5" s="6"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B6" s="9">
+        <v>7253</v>
+      </c>
+      <c r="C6" s="9">
+        <v>7547</v>
+      </c>
+      <c r="D6" s="9">
+        <v>306</v>
+      </c>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" s="9">
+        <v>980</v>
+      </c>
+      <c r="C7" s="9">
+        <v>7648</v>
+      </c>
+      <c r="D7" s="9">
+        <v>205</v>
+      </c>
+      <c r="E7" s="6"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="6"/>
+      <c r="B8" s="8">
+        <f>SUM(B4:B7)</f>
+        <v>8585.82</v>
+      </c>
+      <c r="C8" s="9">
+        <v>7750</v>
+      </c>
+      <c r="D8" s="9">
+        <v>103</v>
+      </c>
+      <c r="E8" s="6"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="10">
+        <f>SUM(C3:C8)</f>
+        <v>44996</v>
+      </c>
+      <c r="D9" s="10">
+        <f>SUM(D3:D8)</f>
+        <v>2502</v>
+      </c>
+      <c r="E9" s="7">
+        <f>C9+D9</f>
+        <v>47498</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>164</v>
+      </c>
+      <c r="B13" t="s">
+        <v>165</v>
+      </c>
+      <c r="E13" t="s">
+        <v>173</v>
+      </c>
+      <c r="F13" t="s">
+        <v>174</v>
+      </c>
+      <c r="H13" t="s">
+        <v>175</v>
+      </c>
+      <c r="I13" t="s">
+        <v>176</v>
+      </c>
+      <c r="L13" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>166</v>
+      </c>
+      <c r="F14" t="s">
+        <v>181</v>
+      </c>
+      <c r="I14" t="s">
+        <v>177</v>
+      </c>
+      <c r="L14" t="s">
+        <v>176</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
souce lab framework created using github copilot agent and mcp
</commit_message>
<xml_diff>
--- a/Playwright_master.xlsx
+++ b/Playwright_master.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="188">
   <si>
     <t xml:space="preserve">Error </t>
   </si>
@@ -752,12 +752,35 @@
   <si>
     <t>page.$$</t>
   </si>
+  <si>
+    <t>.toBe(true)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">value must be exactly </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>true</t>
+    </r>
+  </si>
+  <si>
+    <t>.toBeTruthy()</t>
+  </si>
+  <si>
+    <t>value can be any truthy value</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -820,6 +843,12 @@
       <color rgb="FF001080"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1963,6 +1992,22 @@
         <v>182</v>
       </c>
     </row>
+    <row r="63" spans="2:7" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="B63" t="s">
+        <v>184</v>
+      </c>
+      <c r="C63" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>186</v>
+      </c>
+      <c r="C64" t="s">
+        <v>187</v>
+      </c>
+    </row>
     <row r="68" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C68" s="6"/>
       <c r="D68" s="6"/>

</xml_diff>

<commit_message>
changes done by Copilot for smooth execution
</commit_message>
<xml_diff>
--- a/Playwright_master.xlsx
+++ b/Playwright_master.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010" activeTab="2"/>
+    <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="CommonError&amp;sloution" sheetId="1" r:id="rId1"/>
@@ -13,6 +13,7 @@
     <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="144525"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -261,9 +262,6 @@
     <t>page.frameLocator("Locator")</t>
   </si>
   <si>
-    <t>used to get fream from locator</t>
-  </si>
-  <si>
     <t>#shopping tbody tr:nth-child(2) td:nth-child(1)</t>
   </si>
   <si>
@@ -407,12 +405,6 @@
     <t>to click on specific locator</t>
   </si>
   <si>
-    <t>locator.Click()</t>
-  </si>
-  <si>
-    <t>locator.Click({button:'right'})</t>
-  </si>
-  <si>
     <t>to right click</t>
   </si>
   <si>
@@ -453,12 +445,6 @@
   </si>
   <si>
     <t>used to work with keyboard</t>
-  </si>
-  <si>
-    <t>page.keyboared.press("btn to click" )</t>
-  </si>
-  <si>
-    <t>press enter ofr shift</t>
   </si>
   <si>
     <t xml:space="preserve"> Error: keyboard.press: Unknown key: "control"</t>
@@ -774,6 +760,21 @@
   </si>
   <si>
     <t>value can be any truthy value</t>
+  </si>
+  <si>
+    <t>used to get frame from locator</t>
+  </si>
+  <si>
+    <t>page.locator.Click({button:'right'})</t>
+  </si>
+  <si>
+    <t>page.locator.Click()</t>
+  </si>
+  <si>
+    <t>page.keyboard.press("btn to click" )</t>
+  </si>
+  <si>
+    <t>press enter of shift</t>
   </si>
 </sst>
 </file>
@@ -1279,66 +1280,66 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" t="s">
         <v>75</v>
-      </c>
-      <c r="C5" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" t="s">
         <v>77</v>
-      </c>
-      <c r="C6" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C8" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C9" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C10" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C11" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="90" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="C12" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -1387,10 +1388,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="C4" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1398,10 +1399,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="C5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1409,10 +1410,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="C6" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -1427,7 +1428,7 @@
   <cols>
     <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="63.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="3" max="3" width="74.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="22.28515625" customWidth="1"/>
     <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
@@ -1665,283 +1666,283 @@
         <v>65</v>
       </c>
       <c r="C21" t="s">
-        <v>66</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" t="s">
         <v>67</v>
-      </c>
-      <c r="C22" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C24" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" t="s">
         <v>73</v>
-      </c>
-      <c r="C25" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
+        <v>78</v>
+      </c>
+      <c r="C26" t="s">
         <v>79</v>
-      </c>
-      <c r="C26" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" t="s">
         <v>81</v>
-      </c>
-      <c r="C27" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" t="s">
         <v>83</v>
-      </c>
-      <c r="C28" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" t="s">
         <v>85</v>
-      </c>
-      <c r="C29" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C30" t="s">
         <v>87</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" s="5" t="s">
         <v>88</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" t="s">
         <v>90</v>
-      </c>
-      <c r="C31" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>93</v>
+        <v>185</v>
       </c>
       <c r="C32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>94</v>
+        <v>184</v>
       </c>
       <c r="C33" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C35" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C36" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C37" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C38" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C40" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C41" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>109</v>
+        <v>186</v>
       </c>
       <c r="C42" t="s">
-        <v>110</v>
+        <v>187</v>
       </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C43" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C44" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C45" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C46" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47" s="5" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C47" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C48" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C49" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="50" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C50" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C51" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C52" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="C53" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C54" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.25">
       <c r="C55" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.25">
       <c r="C56" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="D57" s="6"/>
       <c r="E57" s="6"/>
@@ -1950,10 +1951,10 @@
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D58" s="6"/>
       <c r="E58" s="6"/>
@@ -1962,50 +1963,50 @@
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="C59" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="C60" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="61" spans="2:7" ht="90" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C62" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="63" spans="2:7" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C63" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="64" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C64" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="68" spans="3:7" x14ac:dyDescent="0.25">
@@ -2037,7 +2038,7 @@
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
       <c r="C1" s="12" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D1" s="12"/>
       <c r="E1" s="6"/>
@@ -2046,16 +2047,16 @@
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="9" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="E2" s="6"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="9">
@@ -2068,7 +2069,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B4" s="9">
         <v>299</v>
@@ -2083,7 +2084,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B5" s="9">
         <v>53.82</v>
@@ -2098,7 +2099,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B6" s="9">
         <v>7253</v>
@@ -2113,7 +2114,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B7" s="9">
         <v>980</v>
@@ -2158,39 +2159,39 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B13" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E13" t="s">
+        <v>168</v>
+      </c>
+      <c r="F13" t="s">
+        <v>169</v>
+      </c>
+      <c r="H13" t="s">
+        <v>170</v>
+      </c>
+      <c r="I13" t="s">
+        <v>171</v>
+      </c>
+      <c r="L13" t="s">
         <v>173</v>
-      </c>
-      <c r="F13" t="s">
-        <v>174</v>
-      </c>
-      <c r="H13" t="s">
-        <v>175</v>
-      </c>
-      <c r="I13" t="s">
-        <v>176</v>
-      </c>
-      <c r="L13" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="F14" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="I14" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="L14" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>